<commit_message>
remove readonly from fields
</commit_message>
<xml_diff>
--- a/IND-Damage Assessment of Damaged Industrial Facilities.xlsx
+++ b/IND-Damage Assessment of Damaged Industrial Facilities.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mohammed.shurafa\ArcGIS\My Survey Designs\IND-Damage Assessment of Damaged Industrial Facilities\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0808537-6934-45DE-A791-FCE2FAA11DBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE9B6378-2D6C-4BCA-97CE-C4FA312C1E9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="537" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5247" uniqueCount="1576">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3351" uniqueCount="1576">
   <si>
     <t>type</t>
   </si>
@@ -6040,9 +6040,6 @@
       <c r="D36" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="J36" s="1" t="s">
-        <v>1481</v>
-      </c>
       <c r="K36" s="1" t="s">
         <v>1461</v>
       </c>
@@ -6060,9 +6057,6 @@
       <c r="D37" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="J37" s="1" t="s">
-        <v>1481</v>
-      </c>
       <c r="K37" s="1" t="s">
         <v>1461</v>
       </c>
@@ -6077,9 +6071,6 @@
       <c r="C38" s="15" t="s">
         <v>39</v>
       </c>
-      <c r="J38" s="1" t="s">
-        <v>1481</v>
-      </c>
       <c r="K38" s="1" t="s">
         <v>1461</v>
       </c>
@@ -6109,9 +6100,6 @@
       <c r="I39" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="J39" s="1" t="s">
-        <v>1481</v>
-      </c>
       <c r="K39" s="1" t="s">
         <v>1461</v>
       </c>
@@ -6141,9 +6129,6 @@
       <c r="I40" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="J40" s="1" t="s">
-        <v>1481</v>
-      </c>
       <c r="K40" s="1" t="s">
         <v>1461</v>
       </c>
@@ -6161,9 +6146,6 @@
       <c r="C41" s="15" t="s">
         <v>45</v>
       </c>
-      <c r="J41" s="1" t="s">
-        <v>1481</v>
-      </c>
       <c r="K41" s="1" t="s">
         <v>1461</v>
       </c>
@@ -6178,9 +6160,6 @@
       <c r="C42" s="15" t="s">
         <v>47</v>
       </c>
-      <c r="J42" s="1" t="s">
-        <v>1481</v>
-      </c>
       <c r="K42" s="1" t="s">
         <v>1461</v>
       </c>
@@ -6218,9 +6197,6 @@
       <c r="D44" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="J44" s="1" t="s">
-        <v>1481</v>
-      </c>
       <c r="K44" s="1" t="s">
         <v>1461</v>
       </c>
@@ -6255,9 +6231,6 @@
       <c r="C46" s="15" t="s">
         <v>53</v>
       </c>
-      <c r="J46" s="1" t="s">
-        <v>1481</v>
-      </c>
       <c r="K46" s="1" t="s">
         <v>1461</v>
       </c>
@@ -10095,9 +10068,6 @@
       <c r="C291" s="15" t="s">
         <v>240</v>
       </c>
-      <c r="J291" s="1" t="s">
-        <v>1481</v>
-      </c>
       <c r="K291" s="1" t="s">
         <v>1523</v>
       </c>
@@ -10112,9 +10082,6 @@
       <c r="C292" s="15" t="s">
         <v>241</v>
       </c>
-      <c r="J292" s="1" t="s">
-        <v>1481</v>
-      </c>
       <c r="O292" s="1" t="s">
         <v>1237</v>
       </c>
@@ -10129,9 +10096,6 @@
       <c r="C293" s="15" t="s">
         <v>242</v>
       </c>
-      <c r="J293" s="1" t="s">
-        <v>1481</v>
-      </c>
       <c r="K293" s="1" t="s">
         <v>1523</v>
       </c>
@@ -10146,9 +10110,6 @@
       <c r="C294" s="15" t="s">
         <v>243</v>
       </c>
-      <c r="J294" s="1" t="s">
-        <v>1481</v>
-      </c>
       <c r="K294" s="1" t="s">
         <v>1461</v>
       </c>
@@ -10166,9 +10127,6 @@
       <c r="C295" s="15" t="s">
         <v>244</v>
       </c>
-      <c r="J295" s="1" t="s">
-        <v>1481</v>
-      </c>
       <c r="O295" s="1" t="s">
         <v>1238</v>
       </c>
@@ -10340,9 +10298,6 @@
       <c r="C308" s="15" t="s">
         <v>248</v>
       </c>
-      <c r="J308" s="1" t="s">
-        <v>1481</v>
-      </c>
       <c r="K308" s="1" t="s">
         <v>1461</v>
       </c>
@@ -10357,9 +10312,6 @@
       <c r="C309" s="15" t="s">
         <v>249</v>
       </c>
-      <c r="J309" s="1" t="s">
-        <v>1481</v>
-      </c>
       <c r="K309" s="1" t="s">
         <v>1461</v>
       </c>
@@ -10374,9 +10326,6 @@
       <c r="C310" s="15" t="s">
         <v>250</v>
       </c>
-      <c r="J310" s="1" t="s">
-        <v>1481</v>
-      </c>
       <c r="K310" s="1" t="s">
         <v>1461</v>
       </c>
@@ -10391,9 +10340,6 @@
       <c r="C311" s="15" t="s">
         <v>251</v>
       </c>
-      <c r="J311" s="1" t="s">
-        <v>1481</v>
-      </c>
       <c r="K311" s="1" t="s">
         <v>1461</v>
       </c>
@@ -10408,9 +10354,6 @@
       <c r="C312" s="15" t="s">
         <v>252</v>
       </c>
-      <c r="J312" s="1" t="s">
-        <v>1481</v>
-      </c>
       <c r="K312" s="1" t="s">
         <v>1461</v>
       </c>
@@ -10425,9 +10368,6 @@
       <c r="C313" s="15" t="s">
         <v>253</v>
       </c>
-      <c r="J313" s="1" t="s">
-        <v>1481</v>
-      </c>
       <c r="K313" s="1" t="s">
         <v>1461</v>
       </c>
@@ -10442,9 +10382,6 @@
       <c r="C314" s="15" t="s">
         <v>254</v>
       </c>
-      <c r="J314" s="1" t="s">
-        <v>1481</v>
-      </c>
       <c r="K314" s="1" t="s">
         <v>1461</v>
       </c>
@@ -10500,9 +10437,6 @@
       <c r="C318" s="15" t="s">
         <v>257</v>
       </c>
-      <c r="J318" s="1" t="s">
-        <v>1481</v>
-      </c>
       <c r="K318" s="1" t="s">
         <v>1461</v>
       </c>
@@ -10520,9 +10454,6 @@
       <c r="C319" s="15" t="s">
         <v>258</v>
       </c>
-      <c r="J319" s="1" t="s">
-        <v>1481</v>
-      </c>
       <c r="K319" s="1" t="s">
         <v>1461</v>
       </c>
@@ -10537,9 +10468,6 @@
       <c r="C320" s="15" t="s">
         <v>259</v>
       </c>
-      <c r="J320" s="1" t="s">
-        <v>1481</v>
-      </c>
       <c r="K320" s="1" t="s">
         <v>1461</v>
       </c>
@@ -10554,9 +10482,6 @@
       <c r="C321" s="15" t="s">
         <v>260</v>
       </c>
-      <c r="J321" s="1" t="s">
-        <v>1481</v>
-      </c>
       <c r="K321" s="1" t="s">
         <v>1461</v>
       </c>
@@ -10571,9 +10496,6 @@
       <c r="C322" s="15" t="s">
         <v>261</v>
       </c>
-      <c r="J322" s="1" t="s">
-        <v>1481</v>
-      </c>
       <c r="O322" s="1" t="s">
         <v>1239</v>
       </c>
@@ -10615,9 +10537,6 @@
       <c r="C325" s="15" t="s">
         <v>263</v>
       </c>
-      <c r="J325" s="1" t="s">
-        <v>1481</v>
-      </c>
       <c r="K325" s="1" t="s">
         <v>1461</v>
       </c>
@@ -10632,9 +10551,6 @@
       <c r="C326" s="15" t="s">
         <v>264</v>
       </c>
-      <c r="J326" s="1" t="s">
-        <v>1481</v>
-      </c>
       <c r="K326" s="1" t="s">
         <v>1461</v>
       </c>
@@ -10652,9 +10568,6 @@
       <c r="D327" s="1" t="s">
         <v>266</v>
       </c>
-      <c r="J327" s="1" t="s">
-        <v>1481</v>
-      </c>
       <c r="K327" s="1" t="s">
         <v>1461</v>
       </c>
@@ -10672,9 +10585,6 @@
       <c r="D328" s="1" t="s">
         <v>268</v>
       </c>
-      <c r="J328" s="1" t="s">
-        <v>1481</v>
-      </c>
       <c r="K328" s="1" t="s">
         <v>1461</v>
       </c>
@@ -10726,9 +10636,6 @@
       <c r="I331" s="1" t="s">
         <v>273</v>
       </c>
-      <c r="J331" s="1" t="s">
-        <v>1481</v>
-      </c>
     </row>
     <row r="332" spans="1:15" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A332" s="15" t="s">
@@ -10749,9 +10656,6 @@
       <c r="I332" s="1" t="s">
         <v>273</v>
       </c>
-      <c r="J332" s="1" t="s">
-        <v>1481</v>
-      </c>
     </row>
     <row r="333" spans="1:15" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A333" s="15" t="s">
@@ -10772,9 +10676,6 @@
       <c r="I333" s="1" t="s">
         <v>273</v>
       </c>
-      <c r="J333" s="1" t="s">
-        <v>1481</v>
-      </c>
     </row>
     <row r="334" spans="1:15" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A334" s="15" t="s">
@@ -10795,9 +10696,6 @@
       <c r="I334" s="1" t="s">
         <v>273</v>
       </c>
-      <c r="J334" s="1" t="s">
-        <v>1481</v>
-      </c>
     </row>
     <row r="335" spans="1:15" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A335" s="15" t="s">
@@ -10818,9 +10716,6 @@
       <c r="I335" s="1" t="s">
         <v>273</v>
       </c>
-      <c r="J335" s="1" t="s">
-        <v>1481</v>
-      </c>
     </row>
     <row r="336" spans="1:15" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A336" s="15" t="s">
@@ -10846,9 +10741,6 @@
       <c r="C337" s="15" t="s">
         <v>280</v>
       </c>
-      <c r="J337" s="1" t="s">
-        <v>1481</v>
-      </c>
       <c r="K337" s="1" t="s">
         <v>1461</v>
       </c>
@@ -10863,9 +10755,6 @@
       <c r="C338" s="15" t="s">
         <v>281</v>
       </c>
-      <c r="J338" s="1" t="s">
-        <v>1481</v>
-      </c>
       <c r="K338" s="1" t="s">
         <v>1461</v>
       </c>
@@ -10880,9 +10769,6 @@
       <c r="C339" s="15" t="s">
         <v>282</v>
       </c>
-      <c r="J339" s="1" t="s">
-        <v>1481</v>
-      </c>
       <c r="K339" s="1" t="s">
         <v>1461</v>
       </c>
@@ -10897,9 +10783,6 @@
       <c r="C340" s="15" t="s">
         <v>283</v>
       </c>
-      <c r="J340" s="1" t="s">
-        <v>1481</v>
-      </c>
       <c r="K340" s="1" t="s">
         <v>1461</v>
       </c>
@@ -10914,9 +10797,6 @@
       <c r="C341" s="15" t="s">
         <v>284</v>
       </c>
-      <c r="J341" s="1" t="s">
-        <v>1481</v>
-      </c>
       <c r="K341" s="1" t="s">
         <v>1461</v>
       </c>
@@ -10996,9 +10876,6 @@
       <c r="C347" s="15" t="s">
         <v>289</v>
       </c>
-      <c r="J347" s="1" t="s">
-        <v>1481</v>
-      </c>
       <c r="K347" s="1" t="s">
         <v>1461</v>
       </c>
@@ -11012,9 +10889,6 @@
       </c>
       <c r="C348" s="15" t="s">
         <v>290</v>
-      </c>
-      <c r="J348" s="1" t="s">
-        <v>1481</v>
       </c>
       <c r="K348" s="1" t="s">
         <v>1461</v>

</xml_diff>

<commit_message>
remove readonly from fields 001
</commit_message>
<xml_diff>
--- a/IND-Damage Assessment of Damaged Industrial Facilities.xlsx
+++ b/IND-Damage Assessment of Damaged Industrial Facilities.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mohammed.shurafa\ArcGIS\My Survey Designs\IND-Damage Assessment of Damaged Industrial Facilities\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE9B6378-2D6C-4BCA-97CE-C4FA312C1E9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D30A01E-CACD-4BE8-91D4-A54013D729C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="537" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3351" uniqueCount="1576">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3356" uniqueCount="1576">
   <si>
     <t>type</t>
   </si>
@@ -5838,6 +5838,9 @@
       <c r="I26" s="1" t="s">
         <v>20</v>
       </c>
+      <c r="J26" s="1" t="s">
+        <v>1481</v>
+      </c>
       <c r="K26" s="1" t="s">
         <v>1331</v>
       </c>
@@ -5884,6 +5887,9 @@
       <c r="D28" s="1" t="s">
         <v>27</v>
       </c>
+      <c r="J28" s="1" t="s">
+        <v>1481</v>
+      </c>
       <c r="K28" s="1" t="s">
         <v>1331</v>
       </c>
@@ -5930,6 +5936,9 @@
       <c r="I30" s="1" t="s">
         <v>31</v>
       </c>
+      <c r="J30" s="1" t="s">
+        <v>1481</v>
+      </c>
       <c r="K30" s="1" t="s">
         <v>1331</v>
       </c>
@@ -5953,6 +5962,9 @@
       <c r="I31" s="1" t="s">
         <v>31</v>
       </c>
+      <c r="J31" s="1" t="s">
+        <v>1481</v>
+      </c>
       <c r="K31" s="1" t="s">
         <v>1331</v>
       </c>
@@ -5972,6 +5984,9 @@
       </c>
       <c r="F32" s="1" t="s">
         <v>1325</v>
+      </c>
+      <c r="J32" s="1" t="s">
+        <v>1481</v>
       </c>
       <c r="K32" s="1" t="s">
         <v>1331</v>

</xml_diff>